<commit_message>
Updated description input file GeneticsFile.txt
</commit_message>
<xml_diff>
--- a/doc/Manual/Batchmode/GeneticsFile.xlsx
+++ b/doc/Manual/Batchmode/GeneticsFile.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\s02tp3\github\rs_batch_dev\doc\Manual\Batchmode\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\r01cb24\Documents\TestSoftware\RangeShifter_batch\doc\Manual\Batchmode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9723152-EB43-44A9-8554-3FD79E27FA9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{820F3100-46C0-47A3-B751-3982C2DB0D05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2400" windowWidth="21600" windowHeight="11325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="52">
   <si>
     <t>Simulation</t>
   </si>
@@ -42,12 +42,6 @@
   </si>
   <si>
     <t>OutputGeneValues</t>
-  </si>
-  <si>
-    <t>OutputStartGenetics</t>
-  </si>
-  <si>
-    <t>OutputInterval</t>
   </si>
   <si>
     <t>PatchList</t>
@@ -99,30 +93,12 @@
     <t>VALUES</t>
   </si>
   <si>
-    <t>How frequently to output genetic output, including gene values and neutral statistics.</t>
-  </si>
-  <si>
     <t>Positive integer if any output is TRUE, otherwise either 0 or #.</t>
   </si>
   <si>
     <t>Which patches are to be sampled for output.  Patches can be specified according to their patch number, as per the patch layer in a patch-based model. Or sampled randomly or all patches can be chosen. In a cell-based landscape random is the only option with number of patches (=cells) specified.</t>
   </si>
   <si>
-    <t>OutputFstatsWeirCockerham</t>
-  </si>
-  <si>
-    <t>OutputFstatsWeirHill</t>
-  </si>
-  <si>
-    <t>OutputFStatsWeirHill</t>
-  </si>
-  <si>
-    <t>Calculate F-statistics (including global and per-locus estimates) according to Weir &amp; Cockerham (1984)'s method-of-moments approach. Enables the neutralGenetics and perLocusNeutralGenetics output files.</t>
-  </si>
-  <si>
-    <t>Calculate F-statistics calculated according to the estimators of Weir &amp; Hill (2002), including global estimates corrected for unequal sample sizes, population- (i.e. patch-) specific estimates, and pairwise estimates. Enables the neutralGenetics and pairwisePatchNeutralGenetics output files.</t>
-  </si>
-  <si>
     <t>Output the values of all alleles for all genes of all sampled individuals. Does not output the resulting trait values: mean and SD of dispersal and genetic fitness traits are output in the TraitsXPatch, TraitsXCell and/or TraitsXrow output files. Enables the geneValues output files.</t>
   </si>
   <si>
@@ -157,6 +133,51 @@
   </si>
   <si>
     <t>Semicolon-separated list or "all"</t>
+  </si>
+  <si>
+    <t>OutputGenesStart</t>
+  </si>
+  <si>
+    <t>OutputGenesInterval</t>
+  </si>
+  <si>
+    <t>OutputGlobalFst</t>
+  </si>
+  <si>
+    <t>OutputGlobalFstStart</t>
+  </si>
+  <si>
+    <t>OutputGlobalFstInterval</t>
+  </si>
+  <si>
+    <t>OutputPerLocusFst</t>
+  </si>
+  <si>
+    <t>OutputPairwiseFstInterval</t>
+  </si>
+  <si>
+    <t>OutputPairwiseFstStart</t>
+  </si>
+  <si>
+    <t>OutputPairwiseFst</t>
+  </si>
+  <si>
+    <t>Calculate global F-statistics according to Weir &amp; Cockerham (1984)'s method-of-moments approach. Enables the neutralGenetics output file.</t>
+  </si>
+  <si>
+    <t>Calculate F-statistics per-locus estimates according to Weir &amp; Cockerham (1984)'s method-of-moments approach, only if OutputGlobalFst is true, for the same interval as the global fst. Enables the perLocusNeutralGenetics output files.</t>
+  </si>
+  <si>
+    <t>Calculate pairwise F-statistics according to Weir &amp; Cockerham (1984)'s method-of-moments approach. Enables the pairwisePatchNeutralGenetics output files.</t>
+  </si>
+  <si>
+    <t>How frequently to output global F-statistics output.</t>
+  </si>
+  <si>
+    <t>How frequently to output pairwise F-statistics output.</t>
+  </si>
+  <si>
+    <t>How frequently to output gene values output.</t>
   </si>
 </sst>
 </file>
@@ -208,7 +229,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -268,12 +289,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -286,6 +320,16 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -591,15 +635,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C50"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="2" width="67.28515625" customWidth="1"/>
-    <col min="3" max="3" width="52.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="67.26953125" customWidth="1"/>
+    <col min="3" max="3" width="52.453125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
         <v>1</v>
       </c>
@@ -607,265 +651,321 @@
         <v>2</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="5" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="5" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="54.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="116.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+    <row r="19" spans="1:3" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="3" t="s">
+      <c r="B19" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C15"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C16"/>
-    </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C17"/>
-    </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C18"/>
-    </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C19"/>
-    </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C19" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C20"/>
     </row>
-    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C21"/>
     </row>
-    <row r="22" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C22"/>
     </row>
-    <row r="23" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C23"/>
     </row>
-    <row r="24" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C24"/>
     </row>
-    <row r="25" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C25"/>
     </row>
-    <row r="26" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C26"/>
     </row>
-    <row r="27" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C27"/>
     </row>
-    <row r="28" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C28"/>
     </row>
-    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C29"/>
     </row>
-    <row r="30" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C30"/>
     </row>
-    <row r="31" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C31"/>
     </row>
-    <row r="32" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C32"/>
     </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C33"/>
     </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C34"/>
     </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C35"/>
     </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C36"/>
     </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C37"/>
     </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C38"/>
     </row>
-    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C39"/>
     </row>
-    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C40"/>
     </row>
-    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C41"/>
     </row>
-    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C42"/>
     </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C43"/>
     </row>
-    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C44"/>
     </row>
-    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C45"/>
+    </row>
+    <row r="46" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C46"/>
+    </row>
+    <row r="47" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C47"/>
+    </row>
+    <row r="48" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C48"/>
+    </row>
+    <row r="49" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C49"/>
+    </row>
+    <row r="50" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C50"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:R6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" customWidth="1"/>
+    <col min="3" max="3" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -882,31 +982,46 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="G1" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="H1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K1" t="s">
+        <v>45</v>
+      </c>
+      <c r="L1" t="s">
+        <v>44</v>
+      </c>
+      <c r="M1" t="s">
+        <v>43</v>
+      </c>
+      <c r="N1" t="s">
+        <v>42</v>
+      </c>
+      <c r="O1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="P1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="Q1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="R1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -914,40 +1029,55 @@
         <v>300</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" t="b">
         <v>1</v>
       </c>
-      <c r="F2" t="b">
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>5</v>
+      </c>
+      <c r="K2" t="b">
         <v>1</v>
       </c>
-      <c r="G2" t="b">
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>5</v>
+      </c>
+      <c r="N2" t="b">
         <v>1</v>
       </c>
-      <c r="H2">
+      <c r="O2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2">
+        <v>3</v>
+      </c>
+      <c r="Q2">
+        <v>10</v>
+      </c>
+      <c r="R2">
         <v>0</v>
       </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
-      <c r="J2" t="s">
-        <v>14</v>
-      </c>
-      <c r="K2">
-        <v>3</v>
-      </c>
-      <c r="L2">
-        <v>10</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -955,7 +1085,7 @@
         <v>20</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="D3">
         <v>5.0000000000000001E-3</v>
@@ -963,30 +1093,48 @@
       <c r="E3" t="b">
         <v>1</v>
       </c>
-      <c r="F3" t="b">
+      <c r="F3">
         <v>0</v>
       </c>
-      <c r="G3" t="b">
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K3" t="b">
         <v>1</v>
       </c>
-      <c r="H3">
+      <c r="L3">
         <v>0</v>
       </c>
-      <c r="I3">
+      <c r="M3">
         <v>2</v>
       </c>
-      <c r="J3" t="s">
-        <v>40</v>
-      </c>
-      <c r="K3" t="s">
-        <v>13</v>
-      </c>
-      <c r="L3">
+      <c r="N3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O3" t="s">
+        <v>32</v>
+      </c>
+      <c r="P3" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q3">
         <v>10</v>
       </c>
-      <c r="M3" t="s">
-        <v>41</v>
-      </c>
+      <c r="R3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="C6" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>